<commit_message>
Add thumbnail analysis for two videos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHN5v8daos2wujZ76BPAyH
</commit_message>
<xml_diff>
--- a/youtube-world-history-research/output/video_analysis_sheet_filled.xlsx
+++ b/youtube-world-history-research/output/video_analysis_sheet_filled.xlsx
@@ -570,7 +570,11 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>【未確認】モンゴル騎兵とヨーロッパ（騎士・城）を対比させているか／「なぜ止まった？」系の問いを文字にしているか</t>
+          <t>【構図】上下2段。上の約3分の1が文字、下の約3分の2が絵。絵は合戦の一場面を引きで切り取ったもので、中央〜右下で3〜4騎の甲冑の騎馬武者が馬ごと崩れ落ちている（落馬・前のめりに倒れる馬）。
+【文字】「最強が負けた日」1行7文字。文字帯は高さの約34%（縁取り込み）、横幅の約95%まで広げ、左右の余白はほぼなし。1文字の高さは画像の約3割（漢字1字＝幅の約16%）。字間は詰めている。「最強」と「負けた」の正反対の言葉をぶつけ、誰の話かは文字で明かさない（タイトル側で「モンゴル」と明かす分担）。
+【色】背景は茶色・くすんだ金・暗い緑の古画トーンで全体に暗め。目立つ色は2つだけ：文字の黄色（太いゴシック体＋黒の縁取り）と、人物を囲む赤い縁取り。
+【人物の表情】顔は小さく表情はほぼ読めない。のけぞる体・投げ出された手足・崩れる馬など、体の動きで「負けた瞬間」を見せている。
+【絵の風合い】中世の戦記を描いた写本・絵巻の挿絵風。ペルシア細密画（ミニアチュール）風の可能性が高い（平らな金茶色の背景、点々と描いた草、立体感の少ない線描）。</t>
         </is>
       </c>
     </row>
@@ -621,7 +625,11 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>【未確認】怯えるモンゴル兵と武士の構図か／「狩られる側」など逆転を示す言葉があるか</t>
+          <t>【構図】上下の帯文字で絵をはさむサンドイッチ型。中段は左右の対決構図：左に身を寄せ合って縮こまるモンゴル兵5〜6人（狩られる側）、右に刀を振り上げて左へ突進する日本の武者（狩る側）。武者の進行方向（右→左）がモンゴル兵に向かい、視線が「追う側→追われる側」に流れる。
+【文字】4要素で画面の約半分が文字。①上の帯「モンゴル目線で見る元寇」11文字：高さの約16%・幅の約98%、黄色＋黒縁。②左上の吹き出し「怖い怖い怖い怖い怖」9文字（わざと途中で切る）：白い四角に黒文字、高さ約12%・幅約47%。③右の叫び吹き出し「逃がすかおらあぁぁ」約9文字：白いギザギザ吹き出しに赤文字。④下の帯「トラウマ体験すぎる…」10文字：高さの約20%・幅の約95%で一番大きい、赤＋白縁。主役の帯文字は合計21文字。「〜すぎる…」「おらあぁぁ」「怖い」連打など、ネット口語・マンガのセリフ表現で硬い題材をくだけさせている。
+【色】背景は褐色・セピアの古画トーン。文字は上が黄色・下が赤の強い2色を上下に分け、白い吹き出しが間をつなぐ。モンゴル兵は黄土色・オレンジ系で一塊に、武者は青・赤・金など色数が多くこちらが目立つ。
+【人物の表情】モンゴル兵：目を見開き口を開け、頭を抱える・身をすくめる誇張された恐怖顔（ややコミカル）。武者：目をむき歯をむき出しにした鬼の形相で叫ぶ。文字を読まなくても「怖がる側／襲う側」が一瞬でわかる。
+【絵の風合い】右の武者は江戸の武者絵（浮世絵・錦絵）風（歌川国芳のような躍動感）。左のモンゴル兵は古い合戦絵巻の人物をマンガ的に誇張した描き方。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add thumbnail analysis for all 30 model videos
Thumbnails were fetched by inserting them into a Google Doc and exporting
it as PDF, since the container cannot reach YouTube image hosts directly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHN5v8daos2wujZ76BPAyH
</commit_message>
<xml_diff>
--- a/youtube-world-history-research/output/video_analysis_sheet_filled.xlsx
+++ b/youtube-world-history-research/output/video_analysis_sheet_filled.xlsx
@@ -680,7 +680,11 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>【未確認】凶悪な表情の海賊を大きく置いているか／「バケモン」のような強い言葉を文字にしているか</t>
+          <t>【構図】上の黒帯にタイトル1行、中段は中央の赤い縦線で左右2分割の比較構図、下に横幅いっぱいの大きな吹き出し。左：小舟の上で慌てる大陸側の兵たち、右：小舟で武器を振りかざす倭寇の集団。
+【文字】4要素の会話劇。①上帯「海外から見た倭寇、怖すぎる」13文字：黒帯に黄色、高さ約14%・幅約96%。②左の吹き出し「お前ら何者？」6文字：白地に黒。③右の吹き出し「え、ただのゴロツキだよ？」12文字：黒＋「ただのゴロツキ」だけ赤。④下の大吹き出し「じゃあなんでそんな強ぇんだよ…」15文字：白地に赤、高さ約18%で一番大きい。「問い→とぼけ→ツッコミ」の3段で笑わせる。
+【色】黒帯×黄色、中央の赤線、白い吹き出しに赤文字。絵は青い海と黄土・赤の衣服。
+【人物の表情】左の兵は目と口を開けた驚き・恐怖の顔。右の倭寇は余裕のニヤけ顔で、強さと軽さの落差を見せる。
+【絵の風合い】中国・日本の古い絵巻（倭寇図巻のような合戦絵巻）風の線描に彩色したイラスト。</t>
         </is>
       </c>
     </row>
@@ -731,7 +735,11 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>【未確認】コーラ瓶などの商品を象徴的に大きく使っているか／戦場や兵士との組み合わせがあるか</t>
+          <t>【構図】中央にコカ・コーラの瓶を縦いっぱいに大きく置く三分割。左に瓶でコーラを飲む米兵（ヘルメット姿）、右に1920年代風の女性（ヘッドバンド・真珠のネックレス）。背景に古い看板・木箱・炭酸の泡。吹き出しなし。
+【文字】「コーラの歴史」6文字のみ、上部約3割に横幅いっぱい。「コーラ」は赤〜オレンジの燃えるような立体文字、「の歴史」は金色の立体文字。このチャンネルでは珍しく文字が少ない。
+【色】全体がコーラの琥珀色・茶色と赤・金でまとまっている。
+【人物の表情】兵士も女性も笑顔で瓶から飲んでいる（楽しさ・親しみ）。
+【絵の風合い】1940年代アメリカのヴィンテージ広告ポスター風の写実イラスト（AI生成らしい質感）。※再生数÷登録者数は1.1倍で30本中最低。いつもの「会話劇＋ツッコミ」型を外した回でもある。</t>
         </is>
       </c>
     </row>
@@ -782,7 +790,11 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>【未確認】「総集編」の表示があるか／複数の国や人物をどう並べているか</t>
+          <t>【構図】画面を4分割して異なる「国」の絵を並べ（左上：城壁都市の彩色古地図、右上：工場群の俯瞰、左下：煙の上がる町と兵の列、右下：海上の鉄の要塞〈シーランド公国の写真〉）、その中央を大文字が横断する。人物の吹き出しなし。
+【文字】「実在した異常な国」8文字：赤＋白の縁取り＋黒い影、高さ約24%・幅約95%、画面の真ん中。その下に「11選」白＋黒縁。
+【色】4枚の絵はそれぞれ緑・茶・青の別トーンで、中央の赤い大文字が一番目立つ。
+【人物の表情】人物はほぼなし（左下に小さな兵の列のみ）。
+【絵の風合い】中世の彩色地図・版画風イラストと写真のコラージュ。「凡ミスで滅んだ国3選」と同じテンプレート。</t>
         </is>
       </c>
     </row>
@@ -833,7 +845,11 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>【未確認】城壁にはしごで登る兵士など死地の場面か／「99%」の数字を大きく入れているか</t>
+          <t>【構図】上の黒帯にタイトル、下は黄緑一色の背景に、城壁の上で弓を引く兵（左）と、はしごで城壁を登る兵（右）を対角線上に配置。それぞれに吹き出し。
+【文字】①上帯「先頭の兵士って、何考えてたの？」15文字：黒帯に黄色、高さ約16%・幅いっぱい。②弓兵の吹き出し「●ぬよ？」：赤丸の伏せ字＋赤文字（「死ぬよ？」を想像させる）。③登る兵の吹き出し「ですよね。」：白地に黒。脅しへの冷静な返事でシュールな笑いを作る。
+【色】黒帯×黄色、背景の黄緑ベタがとても目立つ。白い城壁と赤い服、赤い伏せ字。
+【人物の表情】弓兵は狙いを定める真顔、登る兵は無表情で淡々。表情は控えめで、吹き出しのセリフで感情を作っている。
+【絵の風合い】鉛筆の線画に水彩で色をつけた、図鑑・教科書の挿絵のような手描き風イラスト。背景だけ単色のベタ塗り。</t>
         </is>
       </c>
     </row>
@@ -884,7 +900,11 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>【未確認】王や人物の脱力した表情など「しょーもなさ」をどう絵にしているか／「3選」を文字にしているか</t>
+          <t>【構図】画面を4分割（左上：海に浮かぶ山の島、右上：工場群の俯瞰、左下：煙の上がる町と兵の列、右下：山あいの木造集落）し、中央を大文字が横断する。「実在した異常な国11選」と同じテンプレート。
+【文字】「凡ミスで滅んだ国」8文字：赤＋白の縁取り、高さ約22%・幅約95%。その下に「3選」白＋黒縁。
+【色】4枚の絵は青・茶・緑の別トーン、中央の赤い大文字が一番目立つ。
+【人物の表情】人物はほぼなし。
+【絵の風合い】古い彩色版画・油絵風の風景イラスト（AI生成らしい質感）。</t>
         </is>
       </c>
     </row>
@@ -935,7 +955,11 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>【未確認】機関銃と、不満そうな軍人の表情を組み合わせているか</t>
+          <t>【構図】左に縦3行の大きな問い、中央に重機関銃（弾帯・弾薬箱つき）の写真を切り抜いて配置、右端に軍服の将校2人。右下に大きな吹き出し2つ。赤い矢印で文字から機関銃を指す。
+【文字】①「なぜ軍人は／機関銃を／嫌ったのか？」3行15文字：黄色＋黒縁、画面左半分・高さの約半分。②吹き出し「使わねぇよ」5文字：白地に黒。③大吹き出し「●●だから。」：赤丸2つの伏せ字＋赤文字、高さ約25%（答えを隠して続きを見させる）。
+【色】エメラルドグリーンのベタ背景（放射状の模様入り）、黄色の文字、赤い矢印・伏せ字。
+【人物の表情】将校たちは口ひげで、機関銃を見下ろす不機嫌・ふてぶてしい顔。
+【絵の風合い】機関銃は写真の切り抜き、将校は19世紀の新聞挿絵・風刺画風のイラスト。</t>
         </is>
       </c>
     </row>
@@ -986,7 +1010,11 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>【未確認】槍兵の密集陣や、騎士が倒される場面か／「地獄」の言葉を文字にしているか</t>
+          <t>【構図】上の黒帯にタイトル、中段は左から「倒れた騎士」「斧槍を振りかぶる歩兵（赤い縁取り）」「右に密集した槍兵の隊列」と、勢いが右から左へ流れる配置。吹き出し2つ。
+【文字】①上帯「※中世の歩兵、怖すぎ問題」12文字：黒帯に黄色、高さ約15%・幅いっぱい。②騎士の吹き出し「こ、降参…」。③歩兵の吹き出し「じゃ●すね？」：赤丸の伏せ字＋「す」赤（「殺すね？」を想像させる）。降参を無視する冷酷さを会話で見せる。
+【色】淡い緑のベタ背景、鎧の金・青、歩兵を囲む赤い縁取り、赤い伏せ字。
+【人物の表情】騎士は力なく倒れて顔をそむける、歩兵は無表情で淡々と斧を振り下ろす（冷酷さ）。
+【絵の風合い】中世ヨーロッパの彩飾写本の挿絵（ミニアチュール）風。</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1065,11 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>【未確認】ヨーロッパの城壁都市と日本の城下町を並べた対比構図か</t>
+          <t>【構図】中央の赤い縦線で左右2分割。左上に「ヨーロッパ」、右上に「日本」の見出し。左に円形の城壁で囲まれた都市、右に天守を中心とした城下町の俯瞰図。上中央と下に吹き出し。
+【文字】①見出し「ヨーロッパ」5文字・「日本」2文字：黒地に黄色、高さ約10%。②上の吹き出し「なんで壁で囲わないの？」11文字：白地に黒（ヨーロッパ側の問い）。③下の吹き出し「ったく、分かってねぇなぁ…」13文字：白地に赤（日本側の返し）。都市を擬人化した会話劇。
+【色】黒×黄色の見出し、中央の赤線、白い吹き出し。絵は淡い水彩の色。
+【人物の表情】人物なし（都市どうしがしゃべっている設定）。
+【絵の風合い】水彩タッチの鳥瞰図イラスト。</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1120,11 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>【未確認】インドの地図や人の多さを見せているか／「14億」の数字を入れているか</t>
+          <t>【構図】上下の帯文字で風景をはさむサンドイッチ型。中段は、左に夕日の平野、上に雨雲とヒマラヤ山脈、右にインド亜大陸の立体地図（輪郭が緑に光り、北側の山脈が赤い線）。青い矢印でモンスーンの風が山にぶつかる様子を図解。
+【文字】①上「ヒマラヤが創った『帝国』」12文字：金色グラデーションの立体文字、高さ約17%。②下「インド人口大国の理由」10文字：赤＋白縁、高さ約16%。上で謎をかけ、下で中身を示す。
+【色】青い空・黒い雨雲・金色の夕日・緑の地図の高彩度（HDR調）。
+【人物の表情】人物なし。
+【絵の風合い】AI生成の高彩度な風景イラスト＋3Dの地形図。</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1175,11 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>【未確認】3つの国の形を並べて見せているか</t>
+          <t>【構図】上半分は暗い紺の世界地図を背景に中央寄せの文字。下半分を3分割し、チリ（オレンジ）・ノルウェー（青）・ベトナム（緑）の地図をそれぞれ光らせて並べる。
+【文字】①「細長い国では／どう暮らしてる？」2行14文字：黄色＋黒縁、中央、高さ約29%。②小見出し「チリ・ノルウェー・ベトナム」13文字：白。
+【色】紺とグレーの地図に、オレンジ・青・緑の3色の発光。
+【人物の表情】人物なし。
+【絵の風合い】デジタル地図のインフォグラフィック風。※倍率1.5倍と低め。問いが「どう暮らしてる？」とゆるく、「なぜ」の矛盾がない。</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1230,11 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>【未確認】地図上でグリーンランドとデンマークの距離を見せているか</t>
+          <t>【構図】左右2分割。左に衛星写真風のグリーンランド（白い氷床と青い海）、右に北欧の白地図でデンマークを赤く塗る。白い矢印でグリーンランドからデンマークへ結ぶ。
+【文字】①「グリーンランドは／なぜデンマーク領？」2行17文字：白＋「デンマーク領」だけ黄色、黒縁、高さ約30%・幅約70%。②小見出し「いま大国が狙う北極の要衝」12文字：白（時事の関心をつなぐ）。地図上に国名ラベル。
+【色】左は青と白、右はベージュの地図に赤。
+【人物の表情】人物なし。
+【絵の風合い】衛星写真と教科書的な白地図の組み合わせ。</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1285,11 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>【未確認】問題の15km部分を地図で拡大しているか</t>
+          <t>【構図】東アジアの白地図を全面に使い、ロシア沿海州を赤く塗る。中国から日本海へ向かう赤い破線の矢印が、海の手前で止まる。文字は左上に寄せる。
+【文字】①「なぜ奪われた？」7文字：赤＋白縁、高さ約15%。②「中国を塞ぐ『15km』」11文字：白＋「15km」だけ黄色、黒縁。地名（中国・北朝鮮・韓国・日本海・ロシア）は明朝体の小さいラベル。
+【色】ベージュの陸と水色の海の落ち着いた地図に、赤だけで強調。
+【人物の表情】人物なし。
+【絵の風合い】和紙のような質感の古地図風の白地図。</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1340,11 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>【未確認】5か国の地図や国旗を並べているか</t>
+          <t>【構図】中央アジアの立体地図を全面に置き、5か国を色分けして赤く光る国境線で囲む。左下に夕日を背にしたラクダの隊商のシルエット（シルクロードの象徴）。
+【文字】①「なぜ5つに分かれた？」10文字：白＋「5つ」だけ黄色、黒縁、高さ約16%。②小見出し「複雑すぎる国境線の謎」10文字：白＋「国境線」黄色、黒帯。国名ラベルは白。
+【色】茶色の背景に、緑・ベージュ・オレンジ・紫の国と、発光する赤い国境線。
+【人物の表情】人物はシルエットのみ。
+【絵の風合い】3D地形図と、夕景の砂漠のAIイラストの組み合わせ。</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1395,11 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>【未確認】「0.2円」など値段の数字を大きく入れているか／ロシアとアメリカを対比しているか</t>
+          <t>【構図】暗い紺の背景に、左にロシア（赤）、右にアラスカ（金色に発光）と北米（グレー）の地図。中央の金色の矢印に「$7,200,000」と書き、ロシアからアラスカへ「売った」流れを見せる。
+【文字】「アラスカを／ロシアはなぜ売った？」2行13文字：「アラスカ」「ロシア」は黄色、それ以外は白、黒縁、左上、高さ約40%。矢印の中に金額「$7,200,000」。
+【色】紺・赤・金の3色だけ。
+【人物の表情】人物なし。
+【絵の風合い】シンプルなベクターの地図。</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1450,11 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>【未確認】2国の国旗や地図を並べているか</t>
+          <t>【構図】羊皮紙風の古地図に、オランダ（オレンジ）とベルギー（緑）を塗り、国境を赤く光らせる。左上に大きな問い、右下に札。
+【文字】①「なぜ別の国に／なったのか？」2行12文字：1行目は金色、2行目は白の太い明朝体、高さ約38%。②小見出し「言葉も近い、隣同士なのに…」13文字：白＋「隣同士」黄色、黒帯。③右下の札「オランダとベルギーの謎」11文字：金の縁取り。
+【色】ベージュの羊皮紙に、オレンジ・緑と赤い国境。
+【人物の表情】人物なし。
+【絵の風合い】アンティークの古地図・羊皮紙風。</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1505,11 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>【未確認】よく似た北欧の国旗を並べて見せているか</t>
+          <t>【構図】北欧の地図だけを全面に置き、ノルウェー（えんじ）・スウェーデン（青）・フィンランド（水色）・デンマーク（赤）を塗り分けて、国名を白文字で入れる。装飾はほぼなし。
+【文字】「なぜ「一つの国」じゃない？」13文字：黄色の太い明朝体、上部1行、高さ約12%・幅約90%。国名ラベルは白。
+【色】紺の海、白い周辺国、北欧4か国の赤〜青系の4色。
+【人物の表情】人物なし。
+【絵の風合い】ごくシンプルなフラットな地図。※30本中で一番はねた（52.5倍）のに、一番シンプルなサムネ。問いの強さで勝っている。</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1560,11 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>【未確認】半島の地図を2色に塗り分けているか</t>
+          <t>【構図】額縁のように囲んだイベリア半島の地図で、スペイン（赤）とポルトガル（青）の2色だけに塗り分ける。上に1行のタイトル。
+【文字】①上「イベリア半島の「二分割」という歴史的謎」17文字：金色の明朝体、高さ約10%と小さめ。②地図上の国名「スペイン」（金色・大きい）、「ポルトガル」（白）。
+【色】紺の海に赤と青の対比、周りは暗いアンティーク調。
+【人物の表情】人物なし。
+【絵の風合い】フラットな地図を古地図風の暗い額縁に収めた形。※文字は控えめでも30.9倍。2色の対比だけで「なぜ分かれた？」が伝わる。</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1615,11 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>【未確認】2国の国旗や人物を対立させる構図か</t>
+          <t>【構図】中央にドイツ（黄色に発光）とオーストリア（赤に発光）の地図。左右に両国の国旗と名所（左：ブランデンブルク門の夜景、右：湖畔の町と教会）。稲妻のような亀裂で左右を分ける。
+【文字】①「同じ言語、全く違う国」10文字：黄色＋黒縁、高さ約19%・幅いっぱい。②小見出し「ドイツとオーストリアが『赤の他人』になった理由」22文字：白＋「赤の他人」だけ赤、黒帯。
+【色】黒・黄・赤（両国の国旗の色）で統一し、強い発光。
+【人物の表情】人物なし。
+【絵の風合い】AI生成の高彩度な写実イラストと発光する地図。</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1670,11 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔を大きく置いているか／「最期」「53歳」などの文字があるか</t>
+          <t>【構図】中央に人物の胸像（制服姿のゲーリング）、上下を文字の帯ではさむ追伸の定番型。
+【文字】①上「ナチス史上最悪の男」9文字：白、高さ約18%・幅いっぱい。②下「ゲーリングの最期」8文字：赤、高さ約22%。上で人物の「肩書き」、下で「名前＋最期」。
+【色】暗い灰色の背景に、白と赤の2色の文字だけ。
+【人物の表情】正面を見据え、口を結んだ落ち着いた（わずかに笑みのある）顔。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1725,11 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>【未確認】若い女性の顔写真を使っているか／「22歳」「悪魔」の文字があるか</t>
+          <t>【構図】中央に若い女性の顔のアップ、上下を文字の帯ではさむ定番型。他の回より背景が明るい（ベージュの壁）ので顔がよく目立つ。
+【文字】①上「ナチス史上最悪の女」9文字：白、高さ約18%。②下「イルマ・グレーゼの最期」11文字：赤、高さ約18%。「男」ではなく「女」にした意外性。
+【色】ベージュの背景に、白と赤の文字。
+【人物の表情】眉をひそめ、カメラをにらむような不機嫌な目つき。「若い女性」と「最悪」の落差を顔で見せる。※チャンネル内で一番の再生数（29.4倍）。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1780,11 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔と「悪魔」「最期」の文字の組み合わせか</t>
+          <t>【構図】中央に人物の胸像、上下を文字の帯ではさむ定番型。背景の左が明るく右が黒い。
+【文字】①上「ナチス史上最悪の男」9文字：白、高さ約18%。②下「ハイドリヒの最期」8文字：赤、高さ約22%。
+【色】白〜黒のグラデーション背景に、白と赤の文字。
+【人物の表情】やや斜めを向き、冷たく見下ろすような目線。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1835,11 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>【未確認】晩年の顔か／「44日間」「4500万人」の数字を入れているか</t>
+          <t>【構図】中央に人物の胸像、上下を文字の帯ではさむ定番型。文字が他の回より大きい。
+【文字】①上「残酷すぎる44日間」9文字（「すぎる」だけ小さく）：白、高さ約23%。②下「毛沢東の最期」6文字：赤、高さ約29%。肩書きではなく「期間＋残酷」を上に置いた形。
+【色】暗い背景に、白と赤の文字。
+【人物の表情】正面を向いた、穏やかな薄笑い（「残酷」との落差）。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1890,11 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔とスターリンを並べているか</t>
+          <t>【構図】中央に人物の胸像、上下を文字の帯ではさむ定番型。
+【文字】①上「大量虐殺した悪魔」8文字：白、高さ約22%。②下「ベリヤの最期」6文字：赤、高さ約28%。
+【色】暗い背景に、白と赤の文字。
+【人物の表情】丸眼鏡の男が正面を向き、無表情で冷たい目つき。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1945,11 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔と「ヒトラーに殺された」の文字があるか</t>
+          <t>【構図】中央に制帽姿の人物の横顔、上下を文字の帯ではさむ定番型。左の背景に別の白黒写真がうっすら重なる。
+【文字】①上「ナチス最高の天才」8文字：白、高さ約21%。②下「ロンメルの最期」7文字：赤、高さ約23%。他の回の「最悪」ではなく「最高」の英雄枠。
+【色】白黒寄りの背景に、白と赤の文字。
+【人物の表情】横を向いて遠くを見つめる、険しく引き締まった表情。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1904,7 +2000,11 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔と「500万人」の数字を入れているか</t>
+          <t>【構図】中央に制帽姿の人物、上下を文字の帯ではさむ定番型。左端にハーケンクロイツの腕章が見える。
+【文字】①上「ナチスが最も恐れた男」10文字：白、高さ約18%。②下「アイヒマンの最期」8文字：赤、高さ約21%。
+【色】暗い緑灰色の背景に、白と赤の文字。
+【人物の表情】口元に薄笑いを浮かべ、こちらをにらむような表情。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -1955,7 +2055,11 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔と「7日間」「1000万人」の数字があるか</t>
+          <t>【構図】中央に人物の胸像、上下を文字の帯ではさむ定番型。文字がとても大きく、上下で1つの文になっている。
+【文字】①上「スターリンの」6文字：白、高さ約26%。②下「最期の7日間」6文字：赤、高さ約31%（30本中で最大級）。名前＋期間だけの短い文。
+【色】明るめのグレーの背景に、白と赤の文字。
+【人物の表情】口ひげで目を細めた薄笑い（不気味さ）。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2110,11 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>【未確認】人物の顔と「逆さ吊り」「10日間」の文字があるか</t>
+          <t>【構図】中央に軍帽・制服のムッソリーニ、その周りを帽子の兵士や側近が囲む集合写真。上下を文字の帯ではさむ。
+【文字】①上「ムッソリーニの」7文字：白、高さ約25%。②下「最期の10日間」7文字：赤、高さ約28%。スターリンの回と同じ「名前の／最期の○日間」型。
+【色】暗い背景にカラー化した写真、白と赤の文字。
+【人物の表情】ムッソリーニはあごを上げて遠くを見る尊大な顔、周りの男たちは険しい顔。
+【絵の風合い】白黒写真をカラー化した肖像写真。背景は暗い灰色〜黒で周囲を暗くした（ビネット）、映画ポスターのような重い雰囲気。文字はかすれのある極太の毛筆・明朝体。</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2165,11 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>【未確認】ヒトラーの顔と「48時間」の文字があるか</t>
+          <t>【構図】他の9本と違う型。背景を4分割（左上：ヒトラーの顔、右上：女性〈エヴァ〉の白黒写真、左下：紫の稲妻、右下：男の白黒写真）し、四隅に小見出しで動画の中身を予告する。中央に大文字。
+【文字】①中央「ヒトラー」4文字：白＋黒縁。②中央下「最後の48時間」7文字：赤＋白縁、高さ約21%。③四隅の小見出し「2通の遺言書を残す」「突然エヴァと結婚する」「青酸カリで愛犬を毒殺」「ヘルマンを処刑する」（各8〜10文字、白）。
+【色】暗い背景に紫の稲妻、白と赤の文字。
+【人物の表情】ヒトラーは目を見開いた険しい顔、他の人物は白黒の不鮮明な写真。
+【絵の風合い】白黒写真のコラージュに稲妻の効果。チャンネルの初期の回（2025年11月）で、後の「上下帯＋肖像」型に固まる前の形。</t>
         </is>
       </c>
     </row>

</xml_diff>